<commit_message>
Remove reference notations from technique descriptions
</commit_message>
<xml_diff>
--- a/public/F3-v1.xlsx
+++ b/public/F3-v1.xlsx
@@ -559,7 +559,7 @@
   </si>
   <si>
     <t xml:space="preserve">Fraud Actors may compromise cloud accounts that can be used during targeting. Adversaries can use compromised cloud accounts to further their operations, including leveraging cloud storage services such as Dropbox, Microsoft OneDrive, or AWS S3 buckets for Exfiltration to Cloud Storage or to Upload Tools. Cloud accounts can also be used in the acquisition of infrastructure, such as Virtual Private Servers or Serverless infrastructure. Additionally, cloud-based messaging services such as Twilio, SendGrid, AWS End User Messaging, AWS SNS (Simple Notification Service), or AWS SES (Simple Email Service) may be leveraged for spam or Phishing. Compromising cloud accounts may allow adversaries to develop sophisticated capabilities without managing their own servers.
-A variety of methods exist for compromising cloud accounts, such as gathering credentials via Phishing for Information, purchasing credentials from third-party sites, conducting Password Spraying attacks, or attempting to Steal Application Access Tokens.[4] Prior to compromising cloud accounts, adversaries may conduct Reconnaissance to inform decisions about which accounts to compromise to further their operation. In some cases, adversaries may target privileged service provider accounts with the intent of leveraging a Trusted Relationship between service providers and their customers.
+A variety of methods exist for compromising cloud accounts, such as gathering credentials via Phishing for Information, purchasing credentials from third-party sites, conducting Password Spraying attacks, or attempting to Steal Application Access Tokens. Prior to compromising cloud accounts, adversaries may conduct Reconnaissance to inform decisions about which accounts to compromise to further their operation. In some cases, adversaries may target privileged service provider accounts with the intent of leveraging a Trusted Relationship between service providers and their customers.
 </t>
   </si>
   <si>
@@ -666,7 +666,7 @@
     <t>Credentials from Password Stores: Password Managers</t>
   </si>
   <si>
-    <t xml:space="preserve">Fraud actors may acquire user credentials from third-party password managers.[1] Password managers are applications designed to store user credentials, normally in an encrypted database. Credentials are typically accessible after a user provides a master password that unlocks the database. After the database is unlocked, these credentials may be copied to memory. These databases can be stored as files on disk. </t>
+    <t xml:space="preserve">Fraud actors may acquire user credentials from third-party password managers. Password managers are applications designed to store user credentials, normally in an encrypted database. Credentials are typically accessible after a user provides a master password that unlocks the database. After the database is unlocked, these credentials may be copied to memory. These databases can be stored as files on disk. </t>
   </si>
   <si>
     <t>Delete Relevant Emails</t>
@@ -702,9 +702,9 @@
     <t>Email Bombing</t>
   </si>
   <si>
-    <t>Fraud actors may flood targeted email addresses with an overwhelming volume of messages. This may bury legitimate emails in a flood of spam and disrupt business operations.[1][2]
-A fraud actor may accomplish email bombing by leveraging an automated bot to register a targeted address for e-mail lists that do not validate new signups, such as online newsletters. The result can be a wave of thousands of e-mails that effectively overloads the victim’s inbox.[2][3]
-By sending hundreds or thousands of e-mails in quick succession, fraud actors may successfully divert attention away from and bury legitimate messages including security alerts, daily business processes like help desk tickets and client correspondence, or ongoing scams.[3] This behavior can also be used as a tool of harassment.[2]</t>
+    <t>Fraud actors may flood targeted email addresses with an overwhelming volume of messages. This may bury legitimate emails in a flood of spam and disrupt business operations.
+A fraud actor may accomplish email bombing by leveraging an automated bot to register a targeted address for e-mail lists that do not validate new signups, such as online newsletters. The result can be a wave of thousands of e-mails that effectively overloads the victim’s inbox.
+By sending hundreds or thousands of e-mails in quick succession, fraud actors may successfully divert attention away from and bury legitimate messages including security alerts, daily business processes like help desk tickets and client correspondence, or ongoing scams. This behavior can also be used as a tool of harassment.</t>
   </si>
   <si>
     <t>T1672</t>

</xml_diff>

<commit_message>
fix modified date bug
</commit_message>
<xml_diff>
--- a/public/F3-v1.xlsx
+++ b/public/F3-v1.xlsx
@@ -1122,7 +1122,9 @@
         </is>
       </c>
       <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="G19" s="11" t="n">
+        <v>46294.5</v>
+      </c>
     </row>
     <row r="20" ht="64" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
@@ -4071,7 +4073,9 @@
         </is>
       </c>
       <c r="F117" s="25" t="n"/>
-      <c r="G117" s="25" t="n"/>
+      <c r="G117" s="25" t="n">
+        <v>46294.5</v>
+      </c>
     </row>
     <row r="118" ht="64" customHeight="1">
       <c r="A118" s="9" t="inlineStr">

</xml_diff>